<commit_message>
resolved the dependency issues...
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DIPANKAR\IdeaProjects\Naukri Automation\naukri-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DIPANKAR\Downloads\Naukri_Automation\naukri-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Username</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t>d.chakraborty1198@gmail.com</t>
+  </si>
+  <si>
+    <t>hi</t>
   </si>
 </sst>
 </file>
@@ -380,14 +383,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.21875" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -395,12 +398,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F15" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>